<commit_message>
round 3 idc_2025 and c_indice_2025
</commit_message>
<xml_diff>
--- a/data/proc_data/private_data/2025_c_educativo.xlsx
+++ b/data/proc_data/private_data/2025_c_educativo.xlsx
@@ -642,7 +642,7 @@
         <v>2</v>
       </c>
       <c r="AG2">
-        <v>0.5268335577959018</v>
+        <v>0.527</v>
       </c>
       <c r="AH2">
         <v>3</v>
@@ -760,7 +760,7 @@
         <v>1</v>
       </c>
       <c r="AG3">
-        <v>0.2840198990005576</v>
+        <v>0.284</v>
       </c>
       <c r="AH3">
         <v>1</v>
@@ -936,7 +936,7 @@
         <v>2</v>
       </c>
       <c r="AG5">
-        <v>0.4650402373198379</v>
+        <v>0.465</v>
       </c>
       <c r="AH5">
         <v>2</v>
@@ -1054,7 +1054,7 @@
         <v>2</v>
       </c>
       <c r="AG6">
-        <v>0.3807224227512509</v>
+        <v>0.381</v>
       </c>
       <c r="AH6">
         <v>1</v>
@@ -1172,7 +1172,7 @@
         <v>2</v>
       </c>
       <c r="AG7">
-        <v>0.5468749408319875</v>
+        <v>0.547</v>
       </c>
       <c r="AH7">
         <v>3</v>
@@ -1290,7 +1290,7 @@
         <v>2</v>
       </c>
       <c r="AG8">
-        <v>0.5322230432940037</v>
+        <v>0.532</v>
       </c>
       <c r="AH8">
         <v>3</v>
@@ -1408,7 +1408,7 @@
         <v>1</v>
       </c>
       <c r="AG9">
-        <v>0.09867339514506224</v>
+        <v>0.099</v>
       </c>
       <c r="AH9">
         <v>1</v>
@@ -1526,7 +1526,7 @@
         <v>2</v>
       </c>
       <c r="AG10">
-        <v>0.5033197334174075</v>
+        <v>0.503</v>
       </c>
       <c r="AH10">
         <v>2</v>
@@ -1644,7 +1644,7 @@
         <v>2</v>
       </c>
       <c r="AG11">
-        <v>0.4227532582376633</v>
+        <v>0.423</v>
       </c>
       <c r="AH11">
         <v>1</v>
@@ -1762,7 +1762,7 @@
         <v>2</v>
       </c>
       <c r="AG12">
-        <v>0.4327816681081055</v>
+        <v>0.433</v>
       </c>
       <c r="AH12">
         <v>1</v>
@@ -1880,7 +1880,7 @@
         <v>2</v>
       </c>
       <c r="AG13">
-        <v>0.4432432905372893</v>
+        <v>0.443</v>
       </c>
       <c r="AH13">
         <v>1</v>
@@ -1998,7 +1998,7 @@
         <v>1</v>
       </c>
       <c r="AG14">
-        <v>0.3243126172300133</v>
+        <v>0.324</v>
       </c>
       <c r="AH14">
         <v>1</v>
@@ -2326,7 +2326,7 @@
         <v>2</v>
       </c>
       <c r="AG18">
-        <v>0.4788754843582047</v>
+        <v>0.479</v>
       </c>
       <c r="AH18">
         <v>2</v>
@@ -2550,7 +2550,7 @@
         <v>3</v>
       </c>
       <c r="AG20">
-        <v>0.5913190300305384</v>
+        <v>0.591</v>
       </c>
       <c r="AH20">
         <v>4</v>
@@ -2668,7 +2668,7 @@
         <v>2</v>
       </c>
       <c r="AG21">
-        <v>0.5037745101440905</v>
+        <v>0.504</v>
       </c>
       <c r="AH21">
         <v>2</v>
@@ -2871,7 +2871,7 @@
         <v>2</v>
       </c>
       <c r="AG23">
-        <v>0.5077929320306707</v>
+        <v>0.508</v>
       </c>
       <c r="AH23">
         <v>2</v>
@@ -2989,7 +2989,7 @@
         <v>3</v>
       </c>
       <c r="AG24">
-        <v>0.5522082315358137</v>
+        <v>0.552</v>
       </c>
       <c r="AH24">
         <v>3</v>
@@ -3107,7 +3107,7 @@
         <v>2</v>
       </c>
       <c r="AG25">
-        <v>0.5427724095213521</v>
+        <v>0.543</v>
       </c>
       <c r="AH25">
         <v>3</v>
@@ -3429,7 +3429,7 @@
         <v>3</v>
       </c>
       <c r="AG29">
-        <v>0.3807224227512509</v>
+        <v>0.381</v>
       </c>
       <c r="AH29">
         <v>1</v>
@@ -3708,7 +3708,7 @@
         <v>2</v>
       </c>
       <c r="AG32">
-        <v>0.4646457619465154</v>
+        <v>0.465</v>
       </c>
       <c r="AH32">
         <v>2</v>
@@ -3826,7 +3826,7 @@
         <v>3</v>
       </c>
       <c r="AG33">
-        <v>0.6117340072667959</v>
+        <v>0.612</v>
       </c>
       <c r="AH33">
         <v>4</v>
@@ -3944,7 +3944,7 @@
         <v>3</v>
       </c>
       <c r="AG34">
-        <v>0.5384272553912703</v>
+        <v>0.538</v>
       </c>
       <c r="AH34">
         <v>3</v>
@@ -4084,7 +4084,7 @@
         <v>2</v>
       </c>
       <c r="AG36">
-        <v>0.536162775743106</v>
+        <v>0.536</v>
       </c>
       <c r="AH36">
         <v>3</v>
@@ -4202,7 +4202,7 @@
         <v>4</v>
       </c>
       <c r="AG37">
-        <v>0.6496091624024841</v>
+        <v>0.65</v>
       </c>
       <c r="AH37">
         <v>4</v>
@@ -4378,7 +4378,7 @@
         <v>2</v>
       </c>
       <c r="AG39">
-        <v>0.5386698782107167</v>
+        <v>0.539</v>
       </c>
       <c r="AH39">
         <v>3</v>
@@ -4594,7 +4594,7 @@
         <v>2</v>
       </c>
       <c r="AG42">
-        <v>0.5587266979516011</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="AH42">
         <v>4</v>
@@ -4770,7 +4770,7 @@
         <v>2</v>
       </c>
       <c r="AG44">
-        <v>0.47890324757345</v>
+        <v>0.479</v>
       </c>
       <c r="AH44">
         <v>2</v>
@@ -5030,7 +5030,7 @@
         <v>3</v>
       </c>
       <c r="AG49">
-        <v>0.5988403374333702</v>
+        <v>0.599</v>
       </c>
       <c r="AH49">
         <v>4</v>
@@ -5210,7 +5210,7 @@
         <v>2</v>
       </c>
       <c r="AG52">
-        <v>0.4446535356753204</v>
+        <v>0.445</v>
       </c>
       <c r="AH52">
         <v>1</v>
@@ -5350,7 +5350,7 @@
         <v>2</v>
       </c>
       <c r="AG54">
-        <v>0.4780926544040323</v>
+        <v>0.478</v>
       </c>
       <c r="AH54">
         <v>2</v>
@@ -5468,7 +5468,7 @@
         <v>2</v>
       </c>
       <c r="AG55">
-        <v>0.5206724640682264</v>
+        <v>0.521</v>
       </c>
       <c r="AH55">
         <v>3</v>
@@ -5586,7 +5586,7 @@
         <v>3</v>
       </c>
       <c r="AG56">
-        <v>0.5667722176885696</v>
+        <v>0.5669999999999999</v>
       </c>
       <c r="AH56">
         <v>4</v>
@@ -5704,7 +5704,7 @@
         <v>2</v>
       </c>
       <c r="AG57">
-        <v>0.5269092884535616</v>
+        <v>0.527</v>
       </c>
       <c r="AH57">
         <v>3</v>
@@ -5822,7 +5822,7 @@
         <v>2</v>
       </c>
       <c r="AG58">
-        <v>0.4996958307596797</v>
+        <v>0.5</v>
       </c>
       <c r="AH58">
         <v>2</v>
@@ -5940,7 +5940,7 @@
         <v>2</v>
       </c>
       <c r="AG59">
-        <v>0.4677422002607572</v>
+        <v>0.468</v>
       </c>
       <c r="AH59">
         <v>2</v>
@@ -6058,7 +6058,7 @@
         <v>3</v>
       </c>
       <c r="AG60">
-        <v>0.5965697540664776</v>
+        <v>0.597</v>
       </c>
       <c r="AH60">
         <v>4</v>
@@ -6176,7 +6176,7 @@
         <v>3</v>
       </c>
       <c r="AG61">
-        <v>0.5834843348192554</v>
+        <v>0.583</v>
       </c>
       <c r="AH61">
         <v>4</v>
@@ -6294,7 +6294,7 @@
         <v>2</v>
       </c>
       <c r="AG62">
-        <v>0.5527915165997067</v>
+        <v>0.553</v>
       </c>
       <c r="AH62">
         <v>3</v>
@@ -6412,7 +6412,7 @@
         <v>3</v>
       </c>
       <c r="AG63">
-        <v>0.5302492840531985</v>
+        <v>0.53</v>
       </c>
       <c r="AH63">
         <v>3</v>
@@ -6530,7 +6530,7 @@
         <v>3</v>
       </c>
       <c r="AG64">
-        <v>0.6003681029995703</v>
+        <v>0.6</v>
       </c>
       <c r="AH64">
         <v>4</v>
@@ -6648,7 +6648,7 @@
         <v>3</v>
       </c>
       <c r="AG65">
-        <v>0.5485463424770612</v>
+        <v>0.549</v>
       </c>
       <c r="AH65">
         <v>3</v>
@@ -6766,7 +6766,7 @@
         <v>3</v>
       </c>
       <c r="AG66">
-        <v>0.5250375085430841</v>
+        <v>0.525</v>
       </c>
       <c r="AH66">
         <v>3</v>
@@ -6884,7 +6884,7 @@
         <v>3</v>
       </c>
       <c r="AG67">
-        <v>0.5649775523062393</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="AH67">
         <v>4</v>
@@ -7002,7 +7002,7 @@
         <v>3</v>
       </c>
       <c r="AG68">
-        <v>0.5530914676344948</v>
+        <v>0.553</v>
       </c>
       <c r="AH68">
         <v>3</v>
@@ -7120,7 +7120,7 @@
         <v>2</v>
       </c>
       <c r="AG69">
-        <v>0.4854834901478353</v>
+        <v>0.485</v>
       </c>
       <c r="AH69">
         <v>2</v>
@@ -7238,7 +7238,7 @@
         <v>2</v>
       </c>
       <c r="AG70">
-        <v>0.4998097899627528</v>
+        <v>0.5</v>
       </c>
       <c r="AH70">
         <v>2</v>
@@ -7356,7 +7356,7 @@
         <v>2</v>
       </c>
       <c r="AG71">
-        <v>0.4896517023784687</v>
+        <v>0.49</v>
       </c>
       <c r="AH71">
         <v>2</v>
@@ -7474,7 +7474,7 @@
         <v>2</v>
       </c>
       <c r="AG72">
-        <v>0.497003827598341</v>
+        <v>0.497</v>
       </c>
       <c r="AH72">
         <v>2</v>
@@ -7592,7 +7592,7 @@
         <v>2</v>
       </c>
       <c r="AG73">
-        <v>0.4985321319744513</v>
+        <v>0.499</v>
       </c>
       <c r="AH73">
         <v>2</v>
@@ -7710,7 +7710,7 @@
         <v>3</v>
       </c>
       <c r="AG74">
-        <v>0.6315801461280494</v>
+        <v>0.632</v>
       </c>
       <c r="AH74">
         <v>4</v>
@@ -7828,7 +7828,7 @@
         <v>2</v>
       </c>
       <c r="AG75">
-        <v>0.493351620948085</v>
+        <v>0.493</v>
       </c>
       <c r="AH75">
         <v>2</v>
@@ -7946,7 +7946,7 @@
         <v>3</v>
       </c>
       <c r="AG76">
-        <v>0.5260172115517473</v>
+        <v>0.526</v>
       </c>
       <c r="AH76">
         <v>3</v>
@@ -8064,7 +8064,7 @@
         <v>2</v>
       </c>
       <c r="AG77">
-        <v>0.5390086758414747</v>
+        <v>0.539</v>
       </c>
       <c r="AH77">
         <v>3</v>
@@ -8182,7 +8182,7 @@
         <v>3</v>
       </c>
       <c r="AG78">
-        <v>0.5330085698007473</v>
+        <v>0.533</v>
       </c>
       <c r="AH78">
         <v>3</v>
@@ -8300,7 +8300,7 @@
         <v>2</v>
       </c>
       <c r="AG79">
-        <v>0.511469533630613</v>
+        <v>0.511</v>
       </c>
       <c r="AH79">
         <v>2</v>
@@ -8418,7 +8418,7 @@
         <v>3</v>
       </c>
       <c r="AG80">
-        <v>0.5754572629334775</v>
+        <v>0.575</v>
       </c>
       <c r="AH80">
         <v>4</v>
@@ -8536,7 +8536,7 @@
         <v>2</v>
       </c>
       <c r="AG81">
-        <v>0.4584425992471785</v>
+        <v>0.458</v>
       </c>
       <c r="AH81">
         <v>1</v>
@@ -8654,7 +8654,7 @@
         <v>2</v>
       </c>
       <c r="AG82">
-        <v>0.4241145808445107</v>
+        <v>0.424</v>
       </c>
       <c r="AH82">
         <v>1</v>
@@ -8772,7 +8772,7 @@
         <v>3</v>
       </c>
       <c r="AG83">
-        <v>0.5221808581352779</v>
+        <v>0.522</v>
       </c>
       <c r="AH83">
         <v>3</v>
@@ -8890,7 +8890,7 @@
         <v>3</v>
       </c>
       <c r="AG84">
-        <v>0.6970841734400132</v>
+        <v>0.697</v>
       </c>
       <c r="AH84">
         <v>4</v>
@@ -9008,7 +9008,7 @@
         <v>3</v>
       </c>
       <c r="AG85">
-        <v>0.5466379959543105</v>
+        <v>0.547</v>
       </c>
       <c r="AH85">
         <v>3</v>
@@ -9126,7 +9126,7 @@
         <v>2</v>
       </c>
       <c r="AG86">
-        <v>0.5127504679674463</v>
+        <v>0.513</v>
       </c>
       <c r="AH86">
         <v>2</v>
@@ -9244,7 +9244,7 @@
         <v>3</v>
       </c>
       <c r="AG87">
-        <v>0.5950796837319542</v>
+        <v>0.595</v>
       </c>
       <c r="AH87">
         <v>4</v>
@@ -9362,7 +9362,7 @@
         <v>3</v>
       </c>
       <c r="AG88">
-        <v>0.502943668047266</v>
+        <v>0.503</v>
       </c>
       <c r="AH88">
         <v>2</v>
@@ -9480,7 +9480,7 @@
         <v>3</v>
       </c>
       <c r="AG89">
-        <v>0.5569041004340289</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="AH89">
         <v>4</v>
@@ -9598,7 +9598,7 @@
         <v>3</v>
       </c>
       <c r="AG90">
-        <v>0.5262483250757369</v>
+        <v>0.526</v>
       </c>
       <c r="AH90">
         <v>3</v>
@@ -9716,7 +9716,7 @@
         <v>2</v>
       </c>
       <c r="AG91">
-        <v>0.2378175820974486</v>
+        <v>0.238</v>
       </c>
       <c r="AH91">
         <v>1</v>
@@ -9834,7 +9834,7 @@
         <v>3</v>
       </c>
       <c r="AG92">
-        <v>0.5355253768106627</v>
+        <v>0.536</v>
       </c>
       <c r="AH92">
         <v>3</v>
@@ -9952,7 +9952,7 @@
         <v>2</v>
       </c>
       <c r="AG93">
-        <v>0.4957614359781685</v>
+        <v>0.496</v>
       </c>
       <c r="AH93">
         <v>2</v>
@@ -10070,7 +10070,7 @@
         <v>2</v>
       </c>
       <c r="AG94">
-        <v>0.4980548182354254</v>
+        <v>0.498</v>
       </c>
       <c r="AH94">
         <v>2</v>
@@ -10188,7 +10188,7 @@
         <v>3</v>
       </c>
       <c r="AG95">
-        <v>0.5758339853776496</v>
+        <v>0.576</v>
       </c>
       <c r="AH95">
         <v>4</v>
@@ -10306,7 +10306,7 @@
         <v>3</v>
       </c>
       <c r="AG96">
-        <v>0.5450629895031235</v>
+        <v>0.545</v>
       </c>
       <c r="AH96">
         <v>3</v>
@@ -10424,7 +10424,7 @@
         <v>2</v>
       </c>
       <c r="AG97">
-        <v>0.3355945783342608</v>
+        <v>0.336</v>
       </c>
       <c r="AH97">
         <v>1</v>
@@ -10542,7 +10542,7 @@
         <v>3</v>
       </c>
       <c r="AG98">
-        <v>0.5966913924611325</v>
+        <v>0.597</v>
       </c>
       <c r="AH98">
         <v>4</v>
@@ -10851,7 +10851,7 @@
         <v>3</v>
       </c>
       <c r="AG101">
-        <v>0.5817920406536182</v>
+        <v>0.582</v>
       </c>
       <c r="AH101">
         <v>4</v>
@@ -10969,7 +10969,7 @@
         <v>3</v>
       </c>
       <c r="AG102">
-        <v>0.5003112104562749</v>
+        <v>0.5</v>
       </c>
       <c r="AH102">
         <v>2</v>
@@ -11087,7 +11087,7 @@
         <v>2</v>
       </c>
       <c r="AG103">
-        <v>0.3280732709314291</v>
+        <v>0.328</v>
       </c>
       <c r="AH103">
         <v>1</v>
@@ -11205,7 +11205,7 @@
         <v>3</v>
       </c>
       <c r="AG104">
-        <v>0.6214042596418652</v>
+        <v>0.621</v>
       </c>
       <c r="AH104">
         <v>4</v>
@@ -11323,7 +11323,7 @@
         <v>3</v>
       </c>
       <c r="AG105">
-        <v>0.5883105070694057</v>
+        <v>0.588</v>
       </c>
       <c r="AH105">
         <v>4</v>
@@ -11441,7 +11441,7 @@
         <v>3</v>
       </c>
       <c r="AG106">
-        <v>0.500484779088648</v>
+        <v>0.5</v>
       </c>
       <c r="AH106">
         <v>2</v>
@@ -11733,7 +11733,7 @@
         <v>2</v>
       </c>
       <c r="AG110">
-        <v>0.3468765394385083</v>
+        <v>0.347</v>
       </c>
       <c r="AH110">
         <v>1</v>
@@ -11851,7 +11851,7 @@
         <v>2</v>
       </c>
       <c r="AG111">
-        <v>0.4650955247897204</v>
+        <v>0.465</v>
       </c>
       <c r="AH111">
         <v>2</v>
@@ -11969,7 +11969,7 @@
         <v>3</v>
       </c>
       <c r="AG112">
-        <v>0.2227749672917853</v>
+        <v>0.223</v>
       </c>
       <c r="AH112">
         <v>1</v>
@@ -12087,7 +12087,7 @@
         <v>3</v>
       </c>
       <c r="AG113">
-        <v>0.6188971571742546</v>
+        <v>0.619</v>
       </c>
       <c r="AH113">
         <v>4</v>
@@ -12205,7 +12205,7 @@
         <v>3</v>
       </c>
       <c r="AG114">
-        <v>0.605287172350083</v>
+        <v>0.605</v>
       </c>
       <c r="AH114">
         <v>4</v>
@@ -12323,7 +12323,7 @@
         <v>2</v>
       </c>
       <c r="AG115">
-        <v>0.3468765394385083</v>
+        <v>0.347</v>
       </c>
       <c r="AH115">
         <v>1</v>
@@ -12441,7 +12441,7 @@
         <v>2</v>
       </c>
       <c r="AG116">
-        <v>0.4721352358010515</v>
+        <v>0.472</v>
       </c>
       <c r="AH116">
         <v>2</v>
@@ -12559,7 +12559,7 @@
         <v>2</v>
       </c>
       <c r="AG117">
-        <v>0.473029377240549</v>
+        <v>0.473</v>
       </c>
       <c r="AH117">
         <v>2</v>
@@ -12677,7 +12677,7 @@
         <v>2</v>
       </c>
       <c r="AG118">
-        <v>0.5449877764290951</v>
+        <v>0.545</v>
       </c>
       <c r="AH118">
         <v>3</v>
@@ -12795,7 +12795,7 @@
         <v>3</v>
       </c>
       <c r="AG119">
-        <v>0.4968326057824652</v>
+        <v>0.497</v>
       </c>
       <c r="AH119">
         <v>2</v>
@@ -12913,7 +12913,7 @@
         <v>2</v>
       </c>
       <c r="AG120">
-        <v>0.491166884087569</v>
+        <v>0.491</v>
       </c>
       <c r="AH120">
         <v>2</v>
@@ -13031,7 +13031,7 @@
         <v>3</v>
       </c>
       <c r="AG121">
-        <v>0.4980548182354254</v>
+        <v>0.498</v>
       </c>
       <c r="AH121">
         <v>2</v>
@@ -13149,7 +13149,7 @@
         <v>3</v>
       </c>
       <c r="AG122">
-        <v>0.6176436059404494</v>
+        <v>0.618</v>
       </c>
       <c r="AH122">
         <v>4</v>
@@ -13267,7 +13267,7 @@
         <v>3</v>
       </c>
       <c r="AG123">
-        <v>0.5723310746157028</v>
+        <v>0.572</v>
       </c>
       <c r="AH123">
         <v>4</v>
@@ -13541,7 +13541,7 @@
         <v>3</v>
       </c>
       <c r="AG127">
-        <v>0.5555148339608372</v>
+        <v>0.556</v>
       </c>
       <c r="AH127">
         <v>4</v>
@@ -13659,7 +13659,7 @@
         <v>2</v>
       </c>
       <c r="AG128">
-        <v>0.4478356272688261</v>
+        <v>0.448</v>
       </c>
       <c r="AH128">
         <v>1</v>
@@ -13777,7 +13777,7 @@
         <v>3</v>
       </c>
       <c r="AG129">
-        <v>0.5709040527942809</v>
+        <v>0.571</v>
       </c>
       <c r="AH129">
         <v>4</v>
@@ -13895,7 +13895,7 @@
         <v>2</v>
       </c>
       <c r="AG130">
-        <v>0.490887454710374</v>
+        <v>0.491</v>
       </c>
       <c r="AH130">
         <v>2</v>
@@ -14013,7 +14013,7 @@
         <v>3</v>
       </c>
       <c r="AG131">
-        <v>0.6007206642840781</v>
+        <v>0.601</v>
       </c>
       <c r="AH131">
         <v>4</v>
@@ -14131,7 +14131,7 @@
         <v>3</v>
       </c>
       <c r="AG132">
-        <v>0.5773508877109939</v>
+        <v>0.577</v>
       </c>
       <c r="AH132">
         <v>4</v>
@@ -14249,7 +14249,7 @@
         <v>2</v>
       </c>
       <c r="AG133">
-        <v>0.5286414683402744</v>
+        <v>0.529</v>
       </c>
       <c r="AH133">
         <v>3</v>
@@ -14367,7 +14367,7 @@
         <v>3</v>
       </c>
       <c r="AG134">
-        <v>0.5360152991273642</v>
+        <v>0.536</v>
       </c>
       <c r="AH134">
         <v>3</v>
@@ -14485,7 +14485,7 @@
         <v>2</v>
       </c>
       <c r="AG135">
-        <v>0.4235938749473915</v>
+        <v>0.424</v>
       </c>
       <c r="AH135">
         <v>1</v>
@@ -14603,7 +14603,7 @@
         <v>2</v>
       </c>
       <c r="AG136">
-        <v>0.4419673544600234</v>
+        <v>0.442</v>
       </c>
       <c r="AH136">
         <v>1</v>
@@ -14697,7 +14697,7 @@
         <v>2</v>
       </c>
       <c r="AG137">
-        <v>0.3205519635285974</v>
+        <v>0.321</v>
       </c>
       <c r="AH137">
         <v>1</v>
@@ -14812,7 +14812,7 @@
         <v>2</v>
       </c>
       <c r="AG138">
-        <v>0.4403556457308451</v>
+        <v>0.44</v>
       </c>
       <c r="AH138">
         <v>1</v>
@@ -14930,7 +14930,7 @@
         <v>2</v>
       </c>
       <c r="AG139">
-        <v>0.5461911856135482</v>
+        <v>0.546</v>
       </c>
       <c r="AH139">
         <v>3</v>
@@ -15106,7 +15106,7 @@
         <v>2</v>
       </c>
       <c r="AG141">
-        <v>0.3468765394385083</v>
+        <v>0.347</v>
       </c>
       <c r="AH141">
         <v>1</v>
@@ -15309,7 +15309,7 @@
         <v>2</v>
       </c>
       <c r="AG143">
-        <v>0.5034854571398429</v>
+        <v>0.503</v>
       </c>
       <c r="AH143">
         <v>2</v>
@@ -15427,7 +15427,7 @@
         <v>3</v>
       </c>
       <c r="AG144">
-        <v>0.5612338004192117</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="AH144">
         <v>4</v>
@@ -15545,7 +15545,7 @@
         <v>2</v>
       </c>
       <c r="AG145">
-        <v>0.2679028117087754</v>
+        <v>0.268</v>
       </c>
       <c r="AH145">
         <v>1</v>
@@ -15663,7 +15663,7 @@
         <v>2</v>
       </c>
       <c r="AG146">
-        <v>0.3017486950215181</v>
+        <v>0.302</v>
       </c>
       <c r="AH146">
         <v>1</v>
@@ -15781,7 +15781,7 @@
         <v>3</v>
       </c>
       <c r="AG147">
-        <v>0.6633652377839789</v>
+        <v>0.663</v>
       </c>
       <c r="AH147">
         <v>4</v>
@@ -15894,7 +15894,7 @@
         <v>2</v>
       </c>
       <c r="AG148">
-        <v>0.4945043874117284</v>
+        <v>0.495</v>
       </c>
       <c r="AH148">
         <v>2</v>
@@ -16007,7 +16007,7 @@
         <v>2</v>
       </c>
       <c r="AG149">
-        <v>0.5053145149459847</v>
+        <v>0.505</v>
       </c>
       <c r="AH149">
         <v>2</v>
@@ -16173,7 +16173,7 @@
         <v>2</v>
       </c>
       <c r="AG151">
-        <v>0.4709781115852312</v>
+        <v>0.471</v>
       </c>
       <c r="AH151">
         <v>2</v>
@@ -16286,7 +16286,7 @@
         <v>3</v>
       </c>
       <c r="AG152">
-        <v>0.5675419937248124</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="AH152">
         <v>4</v>
@@ -16434,7 +16434,7 @@
         <v>3</v>
       </c>
       <c r="AG154">
-        <v>0.5476954470941146</v>
+        <v>0.548</v>
       </c>
       <c r="AH154">
         <v>3</v>
@@ -16547,7 +16547,7 @@
         <v>2</v>
       </c>
       <c r="AG155">
-        <v>0.5481083816181916</v>
+        <v>0.548</v>
       </c>
       <c r="AH155">
         <v>3</v>
@@ -16660,7 +16660,7 @@
         <v>3</v>
       </c>
       <c r="AG156">
-        <v>0.4525167206873717</v>
+        <v>0.453</v>
       </c>
       <c r="AH156">
         <v>1</v>
@@ -16773,7 +16773,7 @@
         <v>2</v>
       </c>
       <c r="AG157">
-        <v>0.4724284085283783</v>
+        <v>0.472</v>
       </c>
       <c r="AH157">
         <v>2</v>
@@ -16886,7 +16886,7 @@
         <v>2</v>
       </c>
       <c r="AG158">
-        <v>0.2944780978654475</v>
+        <v>0.294</v>
       </c>
       <c r="AH158">
         <v>1</v>
@@ -16957,7 +16957,7 @@
         <v>3</v>
       </c>
       <c r="AG159">
-        <v>0.555592819867088</v>
+        <v>0.556</v>
       </c>
       <c r="AH159">
         <v>4</v>
@@ -17043,7 +17043,7 @@
         <v>2</v>
       </c>
       <c r="AG160">
-        <v>0.3965171682971974</v>
+        <v>0.397</v>
       </c>
       <c r="AH160">
         <v>1</v>
@@ -17153,7 +17153,7 @@
         <v>3</v>
       </c>
       <c r="AG161">
-        <v>0.4434783313936279</v>
+        <v>0.443</v>
       </c>
       <c r="AH161">
         <v>1</v>
@@ -17266,7 +17266,7 @@
         <v>2</v>
       </c>
       <c r="AG162">
-        <v>0.5411313969970978</v>
+        <v>0.541</v>
       </c>
       <c r="AH162">
         <v>3</v>
@@ -17459,7 +17459,7 @@
         <v>3</v>
       </c>
       <c r="AG164">
-        <v>0.578156742075583</v>
+        <v>0.578</v>
       </c>
       <c r="AH164">
         <v>4</v>
@@ -17572,7 +17572,7 @@
         <v>2</v>
       </c>
       <c r="AG165">
-        <v>0.4836703178275098</v>
+        <v>0.484</v>
       </c>
       <c r="AH165">
         <v>2</v>
@@ -17685,7 +17685,7 @@
         <v>3</v>
       </c>
       <c r="AG166">
-        <v>0.5434743635478867</v>
+        <v>0.543</v>
       </c>
       <c r="AH166">
         <v>3</v>
@@ -17798,7 +17798,7 @@
         <v>3</v>
       </c>
       <c r="AG167">
-        <v>0.5477929455234106</v>
+        <v>0.548</v>
       </c>
       <c r="AH167">
         <v>3</v>
@@ -17911,7 +17911,7 @@
         <v>3</v>
       </c>
       <c r="AG168">
-        <v>0.7229419095800932</v>
+        <v>0.723</v>
       </c>
       <c r="AH168">
         <v>4</v>
@@ -18157,7 +18157,7 @@
         <v>3</v>
       </c>
       <c r="AG171">
-        <v>0.5791522092318401</v>
+        <v>0.579</v>
       </c>
       <c r="AH171">
         <v>4</v>
@@ -18270,7 +18270,7 @@
         <v>2</v>
       </c>
       <c r="AG172">
-        <v>0.5635480488508522</v>
+        <v>0.5639999999999999</v>
       </c>
       <c r="AH172">
         <v>4</v>
@@ -18463,7 +18463,7 @@
         <v>3</v>
       </c>
       <c r="AG174">
-        <v>0.5406319584027596</v>
+        <v>0.541</v>
       </c>
       <c r="AH174">
         <v>3</v>
@@ -18576,7 +18576,7 @@
         <v>3</v>
       </c>
       <c r="AG175">
-        <v>0.6050343552945256</v>
+        <v>0.605</v>
       </c>
       <c r="AH175">
         <v>4</v>
@@ -18689,7 +18689,7 @@
         <v>2</v>
       </c>
       <c r="AG176">
-        <v>0.5175616929188986</v>
+        <v>0.518</v>
       </c>
       <c r="AH176">
         <v>3</v>
@@ -18802,7 +18802,7 @@
         <v>2</v>
       </c>
       <c r="AG177">
-        <v>0.4963625240697882</v>
+        <v>0.496</v>
       </c>
       <c r="AH177">
         <v>2</v>
@@ -18915,7 +18915,7 @@
         <v>3</v>
       </c>
       <c r="AG178">
-        <v>0.5314494231039981</v>
+        <v>0.531</v>
       </c>
       <c r="AH178">
         <v>3</v>
@@ -19028,7 +19028,7 @@
         <v>2</v>
       </c>
       <c r="AG179">
-        <v>0.4559354967795679</v>
+        <v>0.456</v>
       </c>
       <c r="AH179">
         <v>1</v>
@@ -19194,7 +19194,7 @@
         <v>2</v>
       </c>
       <c r="AG181">
-        <v>0.4385049983648937</v>
+        <v>0.439</v>
       </c>
       <c r="AH181">
         <v>1</v>
@@ -19307,7 +19307,7 @@
         <v>2</v>
       </c>
       <c r="AG182">
-        <v>0.4879010532416027</v>
+        <v>0.488</v>
       </c>
       <c r="AH182">
         <v>2</v>
@@ -19420,7 +19420,7 @@
         <v>3</v>
       </c>
       <c r="AG183">
-        <v>0.5911590022134569</v>
+        <v>0.591</v>
       </c>
       <c r="AH183">
         <v>4</v>
@@ -19586,7 +19586,7 @@
         <v>2</v>
       </c>
       <c r="AG185">
-        <v>0.4387439370016669</v>
+        <v>0.439</v>
       </c>
       <c r="AH185">
         <v>1</v>
@@ -19699,7 +19699,7 @@
         <v>2</v>
       </c>
       <c r="AG186">
-        <v>0.4890762575232951</v>
+        <v>0.489</v>
       </c>
       <c r="AH186">
         <v>2</v>
@@ -19812,7 +19812,7 @@
         <v>2</v>
       </c>
       <c r="AG187">
-        <v>0.4663267767440064</v>
+        <v>0.466</v>
       </c>
       <c r="AH187">
         <v>2</v>
@@ -19925,7 +19925,7 @@
         <v>1</v>
       </c>
       <c r="AG188">
-        <v>0.3310817938925618</v>
+        <v>0.331</v>
       </c>
       <c r="AH188">
         <v>1</v>
@@ -20038,7 +20038,7 @@
         <v>2</v>
       </c>
       <c r="AG189">
-        <v>0.5093801714977663</v>
+        <v>0.509</v>
       </c>
       <c r="AH189">
         <v>2</v>
@@ -20151,7 +20151,7 @@
         <v>4</v>
       </c>
       <c r="AG190">
-        <v>0.7191812558786774</v>
+        <v>0.719</v>
       </c>
       <c r="AH190">
         <v>4</v>
@@ -20264,7 +20264,7 @@
         <v>3</v>
       </c>
       <c r="AG191">
-        <v>0.5161059560022214</v>
+        <v>0.516</v>
       </c>
       <c r="AH191">
         <v>3</v>
@@ -20377,7 +20377,7 @@
         <v>3</v>
       </c>
       <c r="AG192">
-        <v>0.6176436059404494</v>
+        <v>0.618</v>
       </c>
       <c r="AH192">
         <v>4</v>
@@ -20490,7 +20490,7 @@
         <v>2</v>
       </c>
       <c r="AG193">
-        <v>0.4529725574996645</v>
+        <v>0.453</v>
       </c>
       <c r="AH193">
         <v>1</v>
@@ -20603,7 +20603,7 @@
         <v>3</v>
       </c>
       <c r="AG194">
-        <v>0.5161059560022214</v>
+        <v>0.516</v>
       </c>
       <c r="AH194">
         <v>3</v>
@@ -20796,7 +20796,7 @@
         <v>3</v>
       </c>
       <c r="AG196">
-        <v>0.478499418988063</v>
+        <v>0.478</v>
       </c>
       <c r="AH196">
         <v>2</v>
@@ -20909,7 +20909,7 @@
         <v>1</v>
       </c>
       <c r="AG197">
-        <v>0.1325192784578049</v>
+        <v>0.133</v>
       </c>
       <c r="AH197">
         <v>1</v>
@@ -21022,7 +21022,7 @@
         <v>3</v>
       </c>
       <c r="AG198">
-        <v>0.5363299159076134</v>
+        <v>0.536</v>
       </c>
       <c r="AH198">
         <v>3</v>
@@ -21135,7 +21135,7 @@
         <v>2</v>
       </c>
       <c r="AG199">
-        <v>0.5195601860687072</v>
+        <v>0.52</v>
       </c>
       <c r="AH199">
         <v>3</v>
@@ -21248,7 +21248,7 @@
         <v>2</v>
       </c>
       <c r="AG200">
-        <v>0.4355205195433104</v>
+        <v>0.436</v>
       </c>
       <c r="AH200">
         <v>1</v>
@@ -21414,7 +21414,7 @@
         <v>3</v>
       </c>
       <c r="AG202">
-        <v>0.5130290575192449</v>
+        <v>0.513</v>
       </c>
       <c r="AH202">
         <v>2</v>
@@ -21527,7 +21527,7 @@
         <v>2</v>
       </c>
       <c r="AG203">
-        <v>0.5094695082938405</v>
+        <v>0.509</v>
       </c>
       <c r="AH203">
         <v>2</v>
@@ -21640,7 +21640,7 @@
         <v>2</v>
       </c>
       <c r="AG204">
-        <v>0.4897813800923105</v>
+        <v>0.49</v>
       </c>
       <c r="AH204">
         <v>2</v>
@@ -21753,7 +21753,7 @@
         <v>2</v>
       </c>
       <c r="AG205">
-        <v>0.3841937953987117</v>
+        <v>0.384</v>
       </c>
       <c r="AH205">
         <v>1</v>
@@ -21866,7 +21866,7 @@
         <v>2</v>
       </c>
       <c r="AG206">
-        <v>0.5251315248856195</v>
+        <v>0.525</v>
       </c>
       <c r="AH206">
         <v>3</v>
@@ -21979,7 +21979,7 @@
         <v>2</v>
       </c>
       <c r="AG207">
-        <v>0.3762096383095519</v>
+        <v>0.376</v>
       </c>
       <c r="AH207">
         <v>1</v>
@@ -22092,7 +22092,7 @@
         <v>3</v>
       </c>
       <c r="AG208">
-        <v>0.7236940403203763</v>
+        <v>0.724</v>
       </c>
       <c r="AH208">
         <v>4</v>
@@ -22205,7 +22205,7 @@
         <v>2</v>
       </c>
       <c r="AG209">
-        <v>0.5386698782107165</v>
+        <v>0.539</v>
       </c>
       <c r="AH209">
         <v>3</v>
@@ -22318,7 +22318,7 @@
         <v>3</v>
       </c>
       <c r="AG210">
-        <v>0.5386698782107165</v>
+        <v>0.539</v>
       </c>
       <c r="AH210">
         <v>3</v>
@@ -22431,7 +22431,7 @@
         <v>2</v>
       </c>
       <c r="AG211">
-        <v>0.4935420337937264</v>
+        <v>0.494</v>
       </c>
       <c r="AH211">
         <v>2</v>
@@ -22544,7 +22544,7 @@
         <v>3</v>
       </c>
       <c r="AG212">
-        <v>0.6514894892531921</v>
+        <v>0.651</v>
       </c>
       <c r="AH212">
         <v>4</v>
@@ -22657,7 +22657,7 @@
         <v>3</v>
       </c>
       <c r="AG213">
-        <v>0.5443108587628404</v>
+        <v>0.544</v>
       </c>
       <c r="AH213">
         <v>3</v>
@@ -22770,7 +22770,7 @@
         <v>2</v>
       </c>
       <c r="AG214">
-        <v>0.4860207263908947</v>
+        <v>0.486</v>
       </c>
       <c r="AH214">
         <v>2</v>
@@ -22883,7 +22883,7 @@
         <v>2</v>
       </c>
       <c r="AG215">
-        <v>0.4864594693227265</v>
+        <v>0.486</v>
       </c>
       <c r="AH215">
         <v>2</v>
@@ -22996,7 +22996,7 @@
         <v>2</v>
       </c>
       <c r="AG216">
-        <v>0.4810065214556736</v>
+        <v>0.481</v>
       </c>
       <c r="AH216">
         <v>2</v>
@@ -23109,7 +23109,7 @@
         <v>2</v>
       </c>
       <c r="AG217">
-        <v>0.3678287529178251</v>
+        <v>0.368</v>
       </c>
       <c r="AH217">
         <v>1</v>
@@ -23222,7 +23222,7 @@
         <v>2</v>
       </c>
       <c r="AG218">
-        <v>0.3950337993371946</v>
+        <v>0.395</v>
       </c>
       <c r="AH218">
         <v>1</v>
@@ -23335,7 +23335,7 @@
         <v>3</v>
       </c>
       <c r="AG219">
-        <v>0.5315318221405132</v>
+        <v>0.532</v>
       </c>
       <c r="AH219">
         <v>3</v>
@@ -23448,7 +23448,7 @@
         <v>1</v>
       </c>
       <c r="AG220">
-        <v>0.2829454265144389</v>
+        <v>0.283</v>
       </c>
       <c r="AH220">
         <v>1</v>
@@ -23537,7 +23537,7 @@
         <v>3</v>
       </c>
       <c r="AG221">
-        <v>0.5161059560022214</v>
+        <v>0.516</v>
       </c>
       <c r="AH221">
         <v>3</v>
@@ -23647,7 +23647,7 @@
         <v>1</v>
       </c>
       <c r="AG222">
-        <v>0.3355945783342608</v>
+        <v>0.336</v>
       </c>
       <c r="AH222">
         <v>1</v>
@@ -23760,7 +23760,7 @@
         <v>2</v>
       </c>
       <c r="AG223">
-        <v>0.5058496277256328</v>
+        <v>0.506</v>
       </c>
       <c r="AH223">
         <v>2</v>
@@ -23873,7 +23873,7 @@
         <v>2</v>
       </c>
       <c r="AG224">
-        <v>0.3995256912583302</v>
+        <v>0.4</v>
       </c>
       <c r="AH224">
         <v>1</v>
@@ -23986,7 +23986,7 @@
         <v>2</v>
       </c>
       <c r="AG225">
-        <v>0.5341570937690175</v>
+        <v>0.534</v>
       </c>
       <c r="AH225">
         <v>3</v>
@@ -24099,7 +24099,7 @@
         <v>2</v>
       </c>
       <c r="AG226">
-        <v>0.4758833120653389</v>
+        <v>0.476</v>
       </c>
       <c r="AH226">
         <v>2</v>
@@ -24212,7 +24212,7 @@
         <v>3</v>
       </c>
       <c r="AG227">
-        <v>0.5161059560022215</v>
+        <v>0.516</v>
       </c>
       <c r="AH227">
         <v>3</v>
@@ -24325,7 +24325,7 @@
         <v>2</v>
       </c>
       <c r="AG228">
-        <v>0.5048239948979739</v>
+        <v>0.505</v>
       </c>
       <c r="AH228">
         <v>2</v>
@@ -24438,7 +24438,7 @@
         <v>3</v>
       </c>
       <c r="AG229">
-        <v>0.527387917106469</v>
+        <v>0.527</v>
       </c>
       <c r="AH229">
         <v>3</v>
@@ -24551,7 +24551,7 @@
         <v>2</v>
       </c>
       <c r="AG230">
-        <v>0.3920043838554984</v>
+        <v>0.392</v>
       </c>
       <c r="AH230">
         <v>1</v>
@@ -24664,7 +24664,7 @@
         <v>3</v>
       </c>
       <c r="AG231">
-        <v>0.6138829522390336</v>
+        <v>0.614</v>
       </c>
       <c r="AH231">
         <v>4</v>
@@ -24777,7 +24777,7 @@
         <v>2</v>
       </c>
       <c r="AG232">
-        <v>0.4168246982848431</v>
+        <v>0.417</v>
       </c>
       <c r="AH232">
         <v>1</v>
@@ -24890,7 +24890,7 @@
         <v>3</v>
       </c>
       <c r="AG233">
-        <v>0.5972687209611367</v>
+        <v>0.597</v>
       </c>
       <c r="AH233">
         <v>4</v>
@@ -25003,7 +25003,7 @@
         <v>2</v>
       </c>
       <c r="AG234">
-        <v>0.5322230432940037</v>
+        <v>0.532</v>
       </c>
       <c r="AH234">
         <v>3</v>
@@ -25116,7 +25116,7 @@
         <v>3</v>
       </c>
       <c r="AG235">
-        <v>0.5455698602194013</v>
+        <v>0.546</v>
       </c>
       <c r="AH235">
         <v>3</v>
@@ -25309,7 +25309,7 @@
         <v>2</v>
       </c>
       <c r="AG237">
-        <v>0.4032863449597461</v>
+        <v>0.403</v>
       </c>
       <c r="AH237">
         <v>1</v>
@@ -25419,7 +25419,7 @@
         <v>2</v>
       </c>
       <c r="AG238">
-        <v>0.4709781115852312</v>
+        <v>0.471</v>
       </c>
       <c r="AH238">
         <v>2</v>
@@ -25532,7 +25532,7 @@
         <v>3</v>
       </c>
       <c r="AG239">
-        <v>0.5161059560022214</v>
+        <v>0.516</v>
       </c>
       <c r="AH239">
         <v>3</v>
@@ -25805,7 +25805,7 @@
         <v>3</v>
       </c>
       <c r="AG242">
-        <v>0.5247801645397937</v>
+        <v>0.525</v>
       </c>
       <c r="AH242">
         <v>3</v>
@@ -25918,7 +25918,7 @@
         <v>3</v>
       </c>
       <c r="AG243">
-        <v>0.7417451780871724</v>
+        <v>0.742</v>
       </c>
       <c r="AH243">
         <v>4</v>
@@ -26031,7 +26031,7 @@
         <v>2</v>
       </c>
       <c r="AG244">
-        <v>0.5408820274468435</v>
+        <v>0.541</v>
       </c>
       <c r="AH244">
         <v>3</v>
@@ -26144,7 +26144,7 @@
         <v>2</v>
       </c>
       <c r="AG245">
-        <v>0.425850267168241</v>
+        <v>0.426</v>
       </c>
       <c r="AH245">
         <v>1</v>
@@ -26257,7 +26257,7 @@
         <v>2</v>
       </c>
       <c r="AG246">
-        <v>0.478499418988063</v>
+        <v>0.478</v>
       </c>
       <c r="AH246">
         <v>2</v>
@@ -26370,7 +26370,7 @@
         <v>2</v>
       </c>
       <c r="AG247">
-        <v>0.5725157615234592</v>
+        <v>0.573</v>
       </c>
       <c r="AH247">
         <v>4</v>
@@ -26483,7 +26483,7 @@
         <v>2</v>
       </c>
       <c r="AG248">
-        <v>0.4559354967795679</v>
+        <v>0.456</v>
       </c>
       <c r="AH248">
         <v>1</v>
@@ -26684,7 +26684,7 @@
         <v>2</v>
       </c>
       <c r="AG251">
-        <v>0.5407211438660343</v>
+        <v>0.541</v>
       </c>
       <c r="AH251">
         <v>3</v>
@@ -26797,7 +26797,7 @@
         <v>3</v>
       </c>
       <c r="AG252">
-        <v>0.5538448327360779</v>
+        <v>0.554</v>
       </c>
       <c r="AH252">
         <v>4</v>
@@ -26910,7 +26910,7 @@
         <v>2</v>
       </c>
       <c r="AG253">
-        <v>0.4808498275514478</v>
+        <v>0.481</v>
       </c>
       <c r="AH253">
         <v>2</v>
@@ -27023,7 +27023,7 @@
         <v>3</v>
       </c>
       <c r="AG254">
-        <v>0.5973360759528039</v>
+        <v>0.597</v>
       </c>
       <c r="AH254">
         <v>4</v>
@@ -27136,7 +27136,7 @@
         <v>2</v>
       </c>
       <c r="AG255">
-        <v>0.4709781115852312</v>
+        <v>0.471</v>
       </c>
       <c r="AH255">
         <v>2</v>
@@ -27249,7 +27249,7 @@
         <v>3</v>
       </c>
       <c r="AG256">
-        <v>0.4788128067965143</v>
+        <v>0.479</v>
       </c>
       <c r="AH256">
         <v>2</v>
@@ -27362,7 +27362,7 @@
         <v>3</v>
       </c>
       <c r="AG257">
-        <v>0.6439681818503604</v>
+        <v>0.644</v>
       </c>
       <c r="AH257">
         <v>4</v>
@@ -27451,7 +27451,7 @@
         <v>3</v>
       </c>
       <c r="AG258">
-        <v>0.6740534114616871</v>
+        <v>0.674</v>
       </c>
       <c r="AH258">
         <v>4</v>
@@ -27561,7 +27561,7 @@
         <v>2</v>
       </c>
       <c r="AG259">
-        <v>0.5161059560022214</v>
+        <v>0.516</v>
       </c>
       <c r="AH259">
         <v>3</v>
@@ -27674,7 +27674,7 @@
         <v>3</v>
       </c>
       <c r="AG260">
-        <v>0.5870211400860632</v>
+        <v>0.587</v>
       </c>
       <c r="AH260">
         <v>4</v>
@@ -27766,7 +27766,7 @@
         <v>4</v>
       </c>
       <c r="AG261">
-        <v>0.6921045492284832</v>
+        <v>0.6919999999999999</v>
       </c>
       <c r="AH261">
         <v>4</v>
@@ -27876,7 +27876,7 @@
         <v>3</v>
       </c>
       <c r="AG262">
-        <v>0.5609067870538712</v>
+        <v>0.5610000000000001</v>
       </c>
       <c r="AH262">
         <v>4</v>
@@ -27989,7 +27989,7 @@
         <v>3</v>
       </c>
       <c r="AG263">
-        <v>0.4709781115852312</v>
+        <v>0.471</v>
       </c>
       <c r="AH263">
         <v>2</v>
@@ -28102,7 +28102,7 @@
         <v>3</v>
       </c>
       <c r="AG264">
-        <v>0.5499518393149642</v>
+        <v>0.55</v>
       </c>
       <c r="AH264">
         <v>3</v>
@@ -28215,7 +28215,7 @@
         <v>3</v>
       </c>
       <c r="AG265">
-        <v>0.5734051053041994</v>
+        <v>0.573</v>
       </c>
       <c r="AH265">
         <v>4</v>
@@ -28328,7 +28328,7 @@
         <v>3</v>
       </c>
       <c r="AG266">
-        <v>0.5311485708078849</v>
+        <v>0.531</v>
       </c>
       <c r="AH266">
         <v>3</v>
@@ -28441,7 +28441,7 @@
         <v>3</v>
       </c>
       <c r="AG267">
-        <v>0.578156742075583</v>
+        <v>0.578</v>
       </c>
       <c r="AH267">
         <v>4</v>
@@ -28554,7 +28554,7 @@
         <v>3</v>
       </c>
       <c r="AG268">
-        <v>0.5747721537443087</v>
+        <v>0.575</v>
       </c>
       <c r="AH268">
         <v>4</v>
@@ -28667,7 +28667,7 @@
         <v>3</v>
       </c>
       <c r="AG269">
-        <v>0.5837977226277067</v>
+        <v>0.584</v>
       </c>
       <c r="AH269">
         <v>4</v>
@@ -28780,7 +28780,7 @@
         <v>3</v>
       </c>
       <c r="AG270">
-        <v>0.5048239948979739</v>
+        <v>0.505</v>
       </c>
       <c r="AH270">
         <v>2</v>
@@ -28893,7 +28893,7 @@
         <v>3</v>
       </c>
       <c r="AG271">
-        <v>0.6458485087010682</v>
+        <v>0.646</v>
       </c>
       <c r="AH271">
         <v>4</v>
@@ -29006,7 +29006,7 @@
         <v>3</v>
       </c>
       <c r="AG272">
-        <v>0.5386698782107165</v>
+        <v>0.539</v>
       </c>
       <c r="AH272">
         <v>3</v>
@@ -29172,7 +29172,7 @@
         <v>3</v>
       </c>
       <c r="AG274">
-        <v>0.5904985237684114</v>
+        <v>0.59</v>
       </c>
       <c r="AH274">
         <v>4</v>
@@ -29285,7 +29285,7 @@
         <v>2</v>
       </c>
       <c r="AG275">
-        <v>0.4290736846265976</v>
+        <v>0.429</v>
       </c>
       <c r="AH275">
         <v>1</v>
@@ -29398,7 +29398,7 @@
         <v>3</v>
       </c>
       <c r="AG276">
-        <v>0.5077929320306707</v>
+        <v>0.508</v>
       </c>
       <c r="AH276">
         <v>2</v>
@@ -29511,7 +29511,7 @@
         <v>3</v>
       </c>
       <c r="AG277">
-        <v>0.5213868739659119</v>
+        <v>0.521</v>
       </c>
       <c r="AH277">
         <v>3</v>
@@ -29624,7 +29624,7 @@
         <v>2</v>
       </c>
       <c r="AG278">
-        <v>0.4361065954448298</v>
+        <v>0.436</v>
       </c>
       <c r="AH278">
         <v>1</v>
@@ -29737,7 +29737,7 @@
         <v>3</v>
       </c>
       <c r="AG279">
-        <v>0.6518719286126581</v>
+        <v>0.652</v>
       </c>
       <c r="AH279">
         <v>4</v>
@@ -29850,7 +29850,7 @@
         <v>1</v>
       </c>
       <c r="AG280">
-        <v>0.1144681406910089</v>
+        <v>0.114</v>
       </c>
       <c r="AH280">
         <v>1</v>
@@ -29963,7 +29963,7 @@
         <v>3</v>
       </c>
       <c r="AG281">
-        <v>0.527387917106469</v>
+        <v>0.527</v>
       </c>
       <c r="AH281">
         <v>3</v>
@@ -30076,7 +30076,7 @@
         <v>2</v>
       </c>
       <c r="AG282">
-        <v>0.5123453023008055</v>
+        <v>0.512</v>
       </c>
       <c r="AH282">
         <v>2</v>
@@ -30189,7 +30189,7 @@
         <v>2</v>
       </c>
       <c r="AG283">
-        <v>0.481607397253696</v>
+        <v>0.482</v>
       </c>
       <c r="AH283">
         <v>2</v>
@@ -30302,7 +30302,7 @@
         <v>3</v>
       </c>
       <c r="AG284">
-        <v>0.60682449452253</v>
+        <v>0.607</v>
       </c>
       <c r="AH284">
         <v>4</v>
@@ -30415,7 +30415,7 @@
         <v>2</v>
       </c>
       <c r="AG285">
-        <v>0.2302962746946169</v>
+        <v>0.23</v>
       </c>
       <c r="AH285">
         <v>1</v>
@@ -30528,7 +30528,7 @@
         <v>2</v>
       </c>
       <c r="AG286">
-        <v>0.425850267168241</v>
+        <v>0.426</v>
       </c>
       <c r="AH286">
         <v>1</v>
@@ -30641,7 +30641,7 @@
         <v>3</v>
       </c>
       <c r="AG287">
-        <v>0.5455830799086385</v>
+        <v>0.546</v>
       </c>
       <c r="AH287">
         <v>3</v>
@@ -30754,7 +30754,7 @@
         <v>2</v>
       </c>
       <c r="AG288">
-        <v>0.4385786335422641</v>
+        <v>0.439</v>
       </c>
       <c r="AH288">
         <v>1</v>
@@ -30867,7 +30867,7 @@
         <v>3</v>
       </c>
       <c r="AG289">
-        <v>0.5572224364710348</v>
+        <v>0.5570000000000001</v>
       </c>
       <c r="AH289">
         <v>4</v>
@@ -30980,7 +30980,7 @@
         <v>2</v>
       </c>
       <c r="AG290">
-        <v>0.5631141272699196</v>
+        <v>0.5629999999999999</v>
       </c>
       <c r="AH290">
         <v>4</v>
@@ -31093,7 +31093,7 @@
         <v>3</v>
       </c>
       <c r="AG291">
-        <v>0.5124681994805905</v>
+        <v>0.512</v>
       </c>
       <c r="AH291">
         <v>2</v>
@@ -31206,7 +31206,7 @@
         <v>3</v>
       </c>
       <c r="AG292">
-        <v>0.6038545423685913</v>
+        <v>0.604</v>
       </c>
       <c r="AH292">
         <v>4</v>
@@ -31319,7 +31319,7 @@
         <v>2</v>
       </c>
       <c r="AG293">
-        <v>0.4974698276596495</v>
+        <v>0.497</v>
       </c>
       <c r="AH293">
         <v>2</v>
@@ -31432,7 +31432,7 @@
         <v>3</v>
       </c>
       <c r="AG294">
-        <v>0.6560858437771447</v>
+        <v>0.656</v>
       </c>
       <c r="AH294">
         <v>4</v>
@@ -31545,7 +31545,7 @@
         <v>3</v>
       </c>
       <c r="AG295">
-        <v>0.6030710728474631</v>
+        <v>0.603</v>
       </c>
       <c r="AH295">
         <v>4</v>
@@ -31658,7 +31658,7 @@
         <v>3</v>
       </c>
       <c r="AG296">
-        <v>0.5682850261093664</v>
+        <v>0.5679999999999999</v>
       </c>
       <c r="AH296">
         <v>4</v>
@@ -31771,7 +31771,7 @@
         <v>2</v>
       </c>
       <c r="AG297">
-        <v>0.4446535356753204</v>
+        <v>0.445</v>
       </c>
       <c r="AH297">
         <v>1</v>
@@ -31884,7 +31884,7 @@
         <v>2</v>
       </c>
       <c r="AG298">
-        <v>0.4621487507210375</v>
+        <v>0.462</v>
       </c>
       <c r="AH298">
         <v>1</v>
@@ -31997,7 +31997,7 @@
         <v>3</v>
       </c>
       <c r="AG299">
-        <v>0.534711295367121</v>
+        <v>0.535</v>
       </c>
       <c r="AH299">
         <v>3</v>
@@ -32211,7 +32211,7 @@
         <v>3</v>
       </c>
       <c r="AG301">
-        <v>0.5952009951416775</v>
+        <v>0.595</v>
       </c>
       <c r="AH301">
         <v>4</v>
@@ -32324,7 +32324,7 @@
         <v>3</v>
       </c>
       <c r="AG302">
-        <v>0.4032863449597461</v>
+        <v>0.403</v>
       </c>
       <c r="AH302">
         <v>1</v>
@@ -32437,7 +32437,7 @@
         <v>2</v>
       </c>
       <c r="AG303">
-        <v>0.4551833660392847</v>
+        <v>0.455</v>
       </c>
       <c r="AH303">
         <v>1</v>
@@ -32550,7 +32550,7 @@
         <v>2</v>
       </c>
       <c r="AG304">
-        <v>0.513451376918869</v>
+        <v>0.513</v>
       </c>
       <c r="AH304">
         <v>3</v>
@@ -32663,7 +32663,7 @@
         <v>2</v>
       </c>
       <c r="AG305">
-        <v>0.5215524199835824</v>
+        <v>0.522</v>
       </c>
       <c r="AH305">
         <v>3</v>
@@ -32776,7 +32776,7 @@
         <v>2</v>
       </c>
       <c r="AG306">
-        <v>0.4759923165204525</v>
+        <v>0.476</v>
       </c>
       <c r="AH306">
         <v>2</v>
@@ -32889,7 +32889,7 @@
         <v>3</v>
       </c>
       <c r="AG307">
-        <v>0.5085846485993897</v>
+        <v>0.509</v>
       </c>
       <c r="AH307">
         <v>2</v>
@@ -33055,7 +33055,7 @@
         <v>3</v>
       </c>
       <c r="AG309">
-        <v>0.5296443093273185</v>
+        <v>0.53</v>
       </c>
       <c r="AH309">
         <v>3</v>
@@ -33221,7 +33221,7 @@
         <v>2</v>
       </c>
       <c r="AG311">
-        <v>0.5085846485993897</v>
+        <v>0.509</v>
       </c>
       <c r="AH311">
         <v>2</v>
@@ -33334,7 +33334,7 @@
         <v>2</v>
       </c>
       <c r="AG312">
-        <v>0.4889456792697737</v>
+        <v>0.489</v>
       </c>
       <c r="AH312">
         <v>2</v>
@@ -33447,7 +33447,7 @@
         <v>3</v>
       </c>
       <c r="AG313">
-        <v>0.5490116758896102</v>
+        <v>0.549</v>
       </c>
       <c r="AH313">
         <v>3</v>
@@ -33640,7 +33640,7 @@
         <v>2</v>
       </c>
       <c r="AG315">
-        <v>0.5175123793377103</v>
+        <v>0.518</v>
       </c>
       <c r="AH315">
         <v>3</v>
@@ -33753,7 +33753,7 @@
         <v>2</v>
       </c>
       <c r="AG316">
-        <v>0.3882437301540826</v>
+        <v>0.388</v>
       </c>
       <c r="AH316">
         <v>1</v>
@@ -33866,7 +33866,7 @@
         <v>3</v>
       </c>
       <c r="AG317">
-        <v>0.6108744292779009</v>
+        <v>0.611</v>
       </c>
       <c r="AH317">
         <v>4</v>
@@ -33979,7 +33979,7 @@
         <v>2</v>
       </c>
       <c r="AG318">
-        <v>0.3017486950215181</v>
+        <v>0.302</v>
       </c>
       <c r="AH318">
         <v>1</v>
@@ -34092,7 +34092,7 @@
         <v>2</v>
       </c>
       <c r="AG319">
-        <v>0.2876462436412086</v>
+        <v>0.288</v>
       </c>
       <c r="AH319">
         <v>1</v>
@@ -34205,7 +34205,7 @@
         <v>2</v>
       </c>
       <c r="AG320">
-        <v>0.4133147548301883</v>
+        <v>0.413</v>
       </c>
       <c r="AH320">
         <v>1</v>
@@ -34318,7 +34318,7 @@
         <v>2</v>
       </c>
       <c r="AG321">
-        <v>0.3355945783342608</v>
+        <v>0.336</v>
       </c>
       <c r="AH321">
         <v>1</v>
@@ -34431,7 +34431,7 @@
         <v>3</v>
       </c>
       <c r="AG322">
-        <v>0.522373712171248</v>
+        <v>0.522</v>
       </c>
       <c r="AH322">
         <v>3</v>
@@ -34544,7 +34544,7 @@
         <v>2</v>
       </c>
       <c r="AG323">
-        <v>0.4975239024187549</v>
+        <v>0.498</v>
       </c>
       <c r="AH323">
         <v>2</v>
@@ -34657,7 +34657,7 @@
         <v>1</v>
       </c>
       <c r="AG324">
-        <v>0.1325192784578049</v>
+        <v>0.133</v>
       </c>
       <c r="AH324">
         <v>1</v>
@@ -34770,7 +34770,7 @@
         <v>2</v>
       </c>
       <c r="AG325">
-        <v>0.5386698782107165</v>
+        <v>0.539</v>
       </c>
       <c r="AH325">
         <v>3</v>
@@ -34883,7 +34883,7 @@
         <v>2</v>
       </c>
       <c r="AG326">
-        <v>0.4862240049693496</v>
+        <v>0.486</v>
       </c>
       <c r="AH326">
         <v>2</v>
@@ -34996,7 +34996,7 @@
         <v>2</v>
       </c>
       <c r="AG327">
-        <v>0.2929738363848812</v>
+        <v>0.293</v>
       </c>
       <c r="AH327">
         <v>1</v>
@@ -35109,7 +35109,7 @@
         <v>3</v>
       </c>
       <c r="AG328">
-        <v>0.5409589717681001</v>
+        <v>0.541</v>
       </c>
       <c r="AH328">
         <v>3</v>
@@ -35222,7 +35222,7 @@
         <v>2</v>
       </c>
       <c r="AG329">
-        <v>0.4906305599603721</v>
+        <v>0.491</v>
       </c>
       <c r="AH329">
         <v>2</v>
@@ -35489,7 +35489,7 @@
         <v>2</v>
       </c>
       <c r="AG332">
-        <v>0.2829454265144389</v>
+        <v>0.283</v>
       </c>
       <c r="AH332">
         <v>1</v>
@@ -35602,7 +35602,7 @@
         <v>2</v>
       </c>
       <c r="AG333">
-        <v>0.5197161835555807</v>
+        <v>0.52</v>
       </c>
       <c r="AH333">
         <v>3</v>
@@ -35715,7 +35715,7 @@
         <v>2</v>
       </c>
       <c r="AG334">
-        <v>0.5119080169866875</v>
+        <v>0.512</v>
       </c>
       <c r="AH334">
         <v>2</v>
@@ -35828,7 +35828,7 @@
         <v>2</v>
       </c>
       <c r="AG335">
-        <v>0.3732011153484193</v>
+        <v>0.373</v>
       </c>
       <c r="AH335">
         <v>1</v>
@@ -35941,7 +35941,7 @@
         <v>3</v>
       </c>
       <c r="AG336">
-        <v>0.6140709849241044</v>
+        <v>0.614</v>
       </c>
       <c r="AH336">
         <v>4</v>
@@ -36054,7 +36054,7 @@
         <v>3</v>
       </c>
       <c r="AG337">
-        <v>0.5407382377464953</v>
+        <v>0.541</v>
       </c>
       <c r="AH337">
         <v>3</v>
@@ -36167,7 +36167,7 @@
         <v>2</v>
       </c>
       <c r="AG338">
-        <v>0.4296109208696569</v>
+        <v>0.43</v>
       </c>
       <c r="AH338">
         <v>1</v>
@@ -36333,7 +36333,7 @@
         <v>2</v>
       </c>
       <c r="AG340">
-        <v>0.3726638791053598</v>
+        <v>0.373</v>
       </c>
       <c r="AH340">
         <v>1</v>
@@ -36526,7 +36526,7 @@
         <v>2</v>
       </c>
       <c r="AG342">
-        <v>0.3976453644076222</v>
+        <v>0.398</v>
       </c>
       <c r="AH342">
         <v>1</v>
@@ -36639,7 +36639,7 @@
         <v>3</v>
       </c>
       <c r="AG343">
-        <v>0.4461577971558867</v>
+        <v>0.446</v>
       </c>
       <c r="AH343">
         <v>1</v>
@@ -36752,7 +36752,7 @@
         <v>2</v>
       </c>
       <c r="AG344">
-        <v>0.4168246982848431</v>
+        <v>0.417</v>
       </c>
       <c r="AH344">
         <v>1</v>
@@ -36865,7 +36865,7 @@
         <v>3</v>
       </c>
       <c r="AG345">
-        <v>0.7159578384203209</v>
+        <v>0.716</v>
       </c>
       <c r="AH345">
         <v>4</v>
@@ -36978,7 +36978,7 @@
         <v>3</v>
       </c>
       <c r="AG346">
-        <v>0.5916390856647015</v>
+        <v>0.592</v>
       </c>
       <c r="AH346">
         <v>4</v>

</xml_diff>